<commit_message>
feat(channel-allocation): real capture resources on the Clock tab
The Clock nets tab drops the Instrument / Channel / Status columns.
SE Clock Hz now offers exactly the three capture resources
(DAQM907A TOT + the two U2355A counters) and the Frequency band
became a read-only hardware-derived cell: DAQM907A TOT 0 ~ 100 kHz,
U2355A CTR0 / CTR1 0.1 Hz ~ 6 MHz (a legacy free-text band resets to
a clean state).  The Excel round-trip (Power / Clock sheets, import
validation pools) follows the new column sets and the 8 example
projects were regenerated accordingly.
</commit_message>
<xml_diff>
--- a/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
+++ b/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -883,16 +883,10 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>power_capture_nets</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>VDD_3V3
-VDD_1V8
-VDD_5V</t>
-        </is>
-      </c>
+          <t>power_dont_test</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>text</t>
@@ -909,38 +903,52 @@
       <c r="J12" t="b">
         <v>1</v>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>one power net per line (max 12); passed READ-ONLY to block 04 which cannot modify the selection</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Configure Instruments</t>
+          <t>Parse nets for ICT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>instruments</t>
+          <t>parse_ict</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
+          <t>power_capture_nets</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>VDD_3V3
+VDD_1V8
+VDD_5V</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="b">
         <v>1</v>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>one power net per line (max 12); passed READ-ONLY to block 04 which cannot modify the selection</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -955,35 +963,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>psu_visa</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>TCPIP0::192.168.1.20::inst0</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="b">
         <v>1</v>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Keysight N5747A rack PSU (block03 = the ONLY rack-ATE instrument editor)</t>
-        </is>
-      </c>
+      <c r="K14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -998,12 +990,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>daq_visa</t>
+          <t>psu_visa</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GPIB0::9::INSTR</t>
+          <t>TCPIP0::192.168.1.20::inst0</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1024,7 +1016,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Keysight DAQ973A + DAQM908A/907A</t>
+          <t>Keysight N5747A rack PSU (block03 = the ONLY rack-ATE instrument editor)</t>
         </is>
       </c>
     </row>
@@ -1041,10 +1033,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>dmm_visa</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>daq_visa</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>GPIB0::9::INSTR</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
           <t>str</t>
@@ -1052,7 +1048,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1063,7 +1059,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Keysight DMM (optional)</t>
+          <t>Keysight DAQ973A + DAQM908A/907A</t>
         </is>
       </c>
     </row>
@@ -1080,13 +1076,13 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>channel_alloc</t>
+          <t>dmm_visa</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1102,7 +1098,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>one 'instrument:channel:signal' entry per line</t>
+          <t>Keysight DMM (optional)</t>
         </is>
       </c>
     </row>
@@ -1119,17 +1115,13 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>self_test</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+          <t>channel_alloc</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1143,27 +1135,43 @@
       <c r="J18" t="b">
         <v>1</v>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>one 'instrument:channel:signal' entry per line</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Build Impedance/Voltage/Power rails up sequence</t>
+          <t>Configure Instruments</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>rails</t>
+          <t>instruments</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+          <t>self_test</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -1185,30 +1193,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>on_voltage_v</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>float</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>60</v>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="b">
         <v>1</v>
@@ -1228,12 +1220,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>current_limit_a</t>
+          <t>on_voltage_v</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>5.0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1250,7 +1242,7 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>12.5</v>
+        <v>60</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="b">
@@ -1271,29 +1263,29 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>on_delay_ms</t>
+          <t>current_limit_a</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>60000</v>
+        <v>12.5</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="b">
@@ -1314,12 +1306,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>off_delay_ms</t>
+          <t>on_delay_ms</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1357,17 +1349,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>off_protection</t>
+          <t>off_delay_ms</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1375,8 +1367,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>60000</v>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="b">
         <v>1</v>
@@ -1396,24 +1392,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>sequence</t>
+          <t>off_protection</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>VDD_3V3:0.1
-VDD_1V8:0.2
-VDD_5V:0.3</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1422,11 +1416,7 @@
       <c r="J25" t="b">
         <v>1</v>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>one 'rail:delay_s' entry per line</t>
-        </is>
-      </c>
+      <c r="K25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1441,35 +1431,37 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>voltage_tolerance_pct</t>
+          <t>sequence</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>VDD_3V3:0.1
+VDD_1V8:0.2
+VDD_5V:0.3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>5</v>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="b">
         <v>1</v>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>one 'rail:delay_s' entry per line</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1484,12 +1476,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>impedance_min_ohm</t>
+          <t>voltage_tolerance_pct</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1505,7 +1497,9 @@
       <c r="G27" t="n">
         <v>0</v>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>5</v>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="b">
         <v>1</v>
@@ -1525,17 +1519,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sample_rate_hz</t>
+          <t>impedance_min_ohm</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1544,11 +1538,9 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>1</v>
-      </c>
-      <c r="H28" t="n">
-        <v>250000</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="b">
         <v>1</v>
@@ -1568,17 +1560,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pre_trigger_s</t>
+          <t>sample_rate_hz</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1586,8 +1578,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="n">
+        <v>250000</v>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="b">
         <v>1</v>
@@ -1607,12 +1603,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>post_trigger_s</t>
+          <t>pre_trigger_s</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1646,17 +1642,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>anomaly_policy</t>
+          <t>post_trigger_s</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1666,11 +1662,7 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>stop/warn</t>
-        </is>
-      </c>
+      <c r="I31" t="inlineStr"/>
       <c r="J31" t="b">
         <v>1</v>
       </c>
@@ -1679,25 +1671,41 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Build Clocks</t>
+          <t>Build Impedance/Voltage/Power rails up sequence</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>clocks</t>
+          <t>rails</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
+          <t>anomaly_policy</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>stop/warn</t>
+        </is>
+      </c>
       <c r="J32" t="b">
         <v>1</v>
       </c>
@@ -1716,36 +1724,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>clocks</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>CLK1:32768:2
-CLK2:4000000:2</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="b">
         <v>1</v>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>one 'name:freq_hz:tolerance_pct' per line</t>
-        </is>
-      </c>
+      <c r="K33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1760,35 +1751,36 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>stabilize_ms</t>
+          <t>clocks</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>CLK1:32768:2
+CLK2:4000000:2</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" t="n">
-        <v>10000</v>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="b">
         <v>1</v>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>one 'name:freq_hz:tolerance_pct' per line</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1803,17 +1795,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>drift_check</t>
+          <t>stabilize_ms</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1821,8 +1813,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>10000</v>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="b">
         <v>1</v>
@@ -1842,12 +1838,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>multi_domain_check</t>
+          <t>drift_check</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1871,22 +1867,34 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Build GPIOs</t>
+          <t>Build Clocks</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>gpios</t>
+          <t>clocks</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
+          <t>multi_domain_check</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
@@ -1908,36 +1916,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>groups</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>GPIO0:TP_G0.1:out:none
-GPIO1:TP_G1.1:in:pullup</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="b">
         <v>1</v>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>one 'name:pin:mode:pull' per line</t>
-        </is>
-      </c>
+      <c r="K38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1952,35 +1943,36 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>level_threshold_v</t>
+          <t>groups</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>GPIO0:TP_G0.1:out:none
+GPIO1:TP_G1.1:in:pullup</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" t="n">
-        <v>5</v>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="b">
         <v>1</v>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>one 'name:pin:mode:pull' per line</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1995,17 +1987,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>exception_check</t>
+          <t>level_threshold_v</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2013,8 +2005,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>5</v>
+      </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="b">
         <v>1</v>
@@ -2024,22 +2020,34 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Configure Programmer/Debugger</t>
+          <t>Build GPIOs</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>programmer</t>
+          <t>gpios</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
+          <t>exception_check</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
@@ -2061,31 +2069,15 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>protocol</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>SWD</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>SWD/JTAG</t>
-        </is>
-      </c>
+      <c r="I42" t="inlineStr"/>
       <c r="J42" t="b">
         <v>1</v>
       </c>
@@ -2104,17 +2096,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>speed_khz</t>
+          <t>protocol</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>SWD</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2122,13 +2114,13 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G43" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" t="n">
-        <v>100000</v>
-      </c>
-      <c r="I43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>SWD/JTAG</t>
+        </is>
+      </c>
       <c r="J43" t="b">
         <v>1</v>
       </c>
@@ -2147,12 +2139,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>timeout_ms</t>
+          <t>speed_khz</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2166,10 +2158,10 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="H44" t="n">
-        <v>600000</v>
+        <v>100000</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="b">
@@ -2190,17 +2182,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>flash_address</t>
+          <t>timeout_ms</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>0x0</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2208,8 +2200,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
+      <c r="G45" t="n">
+        <v>100</v>
+      </c>
+      <c r="H45" t="n">
+        <v>600000</v>
+      </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="b">
         <v>1</v>
@@ -2229,17 +2225,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>retries</t>
+          <t>flash_address</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2247,12 +2243,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>10</v>
-      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="b">
         <v>1</v>
@@ -2272,17 +2264,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>log_level</t>
+          <t>retries</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2290,13 +2282,13 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>debug/info/warning/error</t>
-        </is>
-      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>10</v>
+      </c>
+      <c r="I47" t="inlineStr"/>
       <c r="J47" t="b">
         <v>1</v>
       </c>
@@ -2305,25 +2297,41 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Configure Peripherals</t>
+          <t>Configure Programmer/Debugger</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>peripherals</t>
+          <t>programmer</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
+          <t>log_level</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>info</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>debug/info/warning/error</t>
+        </is>
+      </c>
       <c r="J48" t="b">
         <v>1</v>
       </c>
@@ -2342,20 +2350,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>wifi_ssid</t>
+          <t>__module__</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>wifi_password</t>
+          <t>wifi_ssid</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>bt_mac</t>
+          <t>wifi_password</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -2447,17 +2447,13 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>uart_baud</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>115200</t>
-        </is>
-      </c>
+          <t>bt_mac</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2465,12 +2461,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G52" t="n">
-        <v>9600</v>
-      </c>
-      <c r="H52" t="n">
-        <v>921600</v>
-      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="b">
         <v>1</v>
@@ -2490,13 +2482,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>i2c_addr</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr"/>
+          <t>uart_baud</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>115200</t>
+        </is>
+      </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2504,8 +2500,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
+      <c r="G53" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H53" t="n">
+        <v>921600</v>
+      </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="b">
         <v>1</v>
@@ -2525,13 +2525,13 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>spi_speed_hz</t>
+          <t>i2c_addr</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2539,9 +2539,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G54" t="n">
-        <v>1</v>
-      </c>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="b">
@@ -2562,13 +2560,13 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>adc_ref_v</t>
+          <t>spi_speed_hz</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2577,11 +2575,9 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" t="n">
-        <v>10</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="b">
         <v>1</v>
@@ -2601,13 +2597,13 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>init_sequence</t>
+          <t>adc_ref_v</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2615,44 +2611,56 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" t="n">
+        <v>10</v>
+      </c>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="b">
         <v>1</v>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>one init step per line</t>
-        </is>
-      </c>
+      <c r="K56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Parse Func/Interface for FCT</t>
+          <t>Configure Peripherals</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>fct_parse</t>
+          <t>peripherals</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>__module__</t>
+          <t>init_sequence</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="b">
-        <v>0</v>
-      </c>
-      <c r="K57" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>one init step per line</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2667,24 +2675,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>spec_file</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>specs/fct_FRDM-IMX93_placeholder.json</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
@@ -2706,22 +2702,22 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>interfaces</t>
+          <t>spec_file</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>(FCT skipped - ICT-only plan)</t>
+          <t>specs/fct_FRDM-IMX93_placeholder.json</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
@@ -2730,11 +2726,7 @@
       <c r="J59" t="b">
         <v>0</v>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>one interface per line</t>
-        </is>
-      </c>
+      <c r="K59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2749,7 +2741,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>protocols</t>
+          <t>interfaces</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2775,7 +2767,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>one protocol per line</t>
+          <t>one interface per line</t>
         </is>
       </c>
     </row>
@@ -2792,10 +2784,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>custom_checks</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+          <t>protocols</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>(FCT skipped - ICT-only plan)</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>text</t>
@@ -2814,36 +2810,48 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>one check rule per line</t>
+          <t>one protocol per line</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Build Func/Interface for FCT</t>
+          <t>Parse Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>fct_build</t>
+          <t>fct_parse</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>__module__</t>
+          <t>custom_checks</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="b">
         <v>0</v>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>one check rule per line</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2858,35 +2866,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>flow_steps</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>(FCT skipped - ICT-only plan)</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="b">
         <v>0</v>
       </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>one flow step per line</t>
-        </is>
-      </c>
+      <c r="K63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2901,35 +2893,35 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>yield_threshold_pct</t>
+          <t>flow_steps</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>98.0</t>
+          <t>(FCT skipped - ICT-only plan)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G64" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" t="n">
-        <v>100</v>
-      </c>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="b">
         <v>0</v>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>one flow step per line</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2944,17 +2936,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>exception_branch</t>
+          <t>yield_threshold_pct</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>98.0</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2962,13 +2954,13 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>continue/stop</t>
-        </is>
-      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="n">
+        <v>100</v>
+      </c>
+      <c r="I65" t="inlineStr"/>
       <c r="J65" t="b">
         <v>0</v>
       </c>
@@ -2987,13 +2979,17 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>case_link</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
+          <t>exception_branch</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -3003,7 +2999,11 @@
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>continue/stop</t>
+        </is>
+      </c>
       <c r="J66" t="b">
         <v>0</v>
       </c>
@@ -3012,27 +3012,35 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Validate Full Test Sequence</t>
+          <t>Build Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>validate_sequence</t>
+          <t>fct_build</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>__module__</t>
+          <t>case_link</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K67" t="inlineStr"/>
     </row>
@@ -3049,24 +3057,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>resource_conflict_check</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
@@ -3088,12 +3084,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>param_range_check</t>
+          <t>resource_conflict_check</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3127,12 +3123,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>dependency_check</t>
+          <t>param_range_check</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3156,22 +3152,34 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Preview &amp; Export YAML</t>
+          <t>Validate Full Test Sequence</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>preview_export</t>
+          <t>validate_sequence</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
+          <t>dependency_check</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
@@ -3193,35 +3201,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>export_dir</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>config/plans</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="b">
         <v>1</v>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>project config folder for the exported YAML</t>
-        </is>
-      </c>
+      <c r="K72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3236,17 +3228,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>include_disabled</t>
+          <t>export_dir</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>config/plans</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3260,7 +3252,50 @@
       <c r="J73" t="b">
         <v>1</v>
       </c>
-      <c r="K73" t="inlineStr"/>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>project config folder for the exported YAML</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Preview &amp; Export YAML</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>preview_export</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>include_disabled</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr"/>
+      <c r="J74" t="b">
+        <v>1</v>
+      </c>
+      <c r="K74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3273,7 +3308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3289,32 +3324,17 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Instrument</t>
+          <t>Impedance</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Power rails</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Impedance(Yes/No)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Power rails(Yes/No)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Voltage(Yes/No)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>Voltage</t>
         </is>
       </c>
     </row>
@@ -3331,32 +3351,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DAQ973A</t>
+          <t>DAQM908A #1 CH101</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CH01</t>
+          <t>U2355A AI01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>DAQM908A #2 CH201</t>
         </is>
       </c>
     </row>
@@ -3373,32 +3378,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DAQ973A</t>
+          <t>DAQM908A #1 CH102</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CH02</t>
+          <t>U2355A AI02</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>DAQM908A #2 CH202</t>
         </is>
       </c>
     </row>
@@ -3415,32 +3405,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DAQ973A</t>
+          <t>DAQM908A #1 CH103</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CH03</t>
+          <t>U2355A AI03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>DAQM908A #2 CH203</t>
         </is>
       </c>
     </row>
@@ -3455,7 +3430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3471,27 +3446,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Instrument</t>
+          <t>SE Clock Hz</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>SE Clock Hz(Yes/No)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
           <t>Frequency band</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Status</t>
         </is>
       </c>
     </row>
@@ -3508,27 +3468,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DAQ973A</t>
+          <t>DAQM907A TOT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CH09</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>CH1 source: DAQM907A</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>0 ~ 100 kHz</t>
         </is>
       </c>
     </row>
@@ -3545,27 +3490,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DAQ973A</t>
+          <t>U2355A CTR0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CH10</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CH2 source: U2355A</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>0.1 Hz ~ 6 MHz</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(channel-allocation): DAQM907A DIO pool on the GPIO tab
The GPIO nets tab drops the Instrument / Channel / Status / Digital
Input / Digital Output columns and picks the DIO resource directly:
the DIO Channel combo offers exactly the 16 DAQM907A DIO channels -
the U2355A DIO is NOT offered (reserved for the fixture control).
GPIO-row validation needs only test point + DIO channel; the Excel
round-trip follows the 3-column GPIO sheet and the 8 example
projects were regenerated accordingly.
</commit_message>
<xml_diff>
--- a/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
+++ b/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
@@ -3510,7 +3510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3526,27 +3526,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Instrument</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Channel</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Digital Input(HighZ)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Digital Output(No Output)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Status</t>
+          <t>DIO Channel</t>
         </is>
       </c>
     </row>
@@ -3563,27 +3543,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>U2355A</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>CH17</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>HighZ</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>No Output</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>DAQM907A DIO01</t>
         </is>
       </c>
     </row>
@@ -3600,27 +3560,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>U2355A</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>CH18</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>HighZ</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>No Output</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>DAQM907A DIO02</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(power-tree): drop the side panels and the capture-nets feature
The Power Tree page keeps ONLY the interactive topology canvas
(node edit via double-click, zoom / pan / fit): the Power Nodes
summary table and the Audit Log panel are removed (unnecessary) and
the Power Waveform Capture Nets section is deleted entirely - the
power_capture_nets schema field, the block-dialog candidates
plumbing (power_candidates args, power_capture_candidates helper)
and its test module are gone, the 8 example projects no longer
carry the parameter.
</commit_message>
<xml_diff>
--- a/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
+++ b/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K74"/>
+  <dimension ref="A1:K73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -908,47 +908,29 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Parse nets for ICT</t>
+          <t>Configure Instruments</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>parse_ict</t>
+          <t>instruments</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>power_capture_nets</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>VDD_3V3
-VDD_1V8
-VDD_5V</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="b">
         <v>1</v>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>one power net per line (max 12); passed READ-ONLY to block 04 which cannot modify the selection</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -963,19 +945,35 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+          <t>psu_visa</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TCPIP0::192.168.1.20::inst0</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="b">
         <v>1</v>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Keysight N5747A rack PSU (block03 = the ONLY rack-ATE instrument editor)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -990,12 +988,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>psu_visa</t>
+          <t>daq_visa</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>TCPIP0::192.168.1.20::inst0</t>
+          <t>GPIB0::9::INSTR</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1016,7 +1014,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Keysight N5747A rack PSU (block03 = the ONLY rack-ATE instrument editor)</t>
+          <t>Keysight DAQ973A + DAQM908A/907A</t>
         </is>
       </c>
     </row>
@@ -1033,14 +1031,10 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>daq_visa</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>GPIB0::9::INSTR</t>
-        </is>
-      </c>
+          <t>dmm_visa</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>str</t>
@@ -1048,7 +1042,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -1059,7 +1053,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Keysight DAQ973A + DAQM908A/907A</t>
+          <t>Keysight DMM (optional)</t>
         </is>
       </c>
     </row>
@@ -1076,13 +1070,13 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>dmm_visa</t>
+          <t>channel_alloc</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1098,7 +1092,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Keysight DMM (optional)</t>
+          <t>one 'instrument:channel:signal' entry per line</t>
         </is>
       </c>
     </row>
@@ -1115,13 +1109,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>channel_alloc</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>self_test</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1135,43 +1133,27 @@
       <c r="J18" t="b">
         <v>1</v>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>one 'instrument:channel:signal' entry per line</t>
-        </is>
-      </c>
+      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Configure Instruments</t>
+          <t>Build Impedance/Voltage/Power rails up sequence</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>instruments</t>
+          <t>rails</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>self_test</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -1193,14 +1175,30 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+          <t>on_voltage_v</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>60</v>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="b">
         <v>1</v>
@@ -1220,12 +1218,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>on_voltage_v</t>
+          <t>current_limit_a</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1242,7 +1240,7 @@
         <v>0</v>
       </c>
       <c r="H21" t="n">
-        <v>60</v>
+        <v>12.5</v>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="b">
@@ -1263,29 +1261,29 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>current_limit_a</t>
+          <t>on_delay_ms</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G22" t="n">
         <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>12.5</v>
+        <v>60000</v>
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="b">
@@ -1306,12 +1304,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>on_delay_ms</t>
+          <t>off_delay_ms</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>200</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1349,17 +1347,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>off_delay_ms</t>
+          <t>off_protection</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1367,12 +1365,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>60000</v>
-      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="b">
         <v>1</v>
@@ -1392,22 +1386,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>off_protection</t>
+          <t>sequence</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>VDD_3V3:0.1
+VDD_1V8:0.2
+VDD_5V:0.3</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr"/>
@@ -1416,7 +1412,11 @@
       <c r="J25" t="b">
         <v>1</v>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>one 'rail:delay_s' entry per line</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1431,37 +1431,35 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>sequence</t>
+          <t>voltage_tolerance_pct</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>VDD_3V3:0.1
-VDD_1V8:0.2
-VDD_5V:0.3</t>
+          <t>0.1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>5</v>
+      </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="b">
         <v>1</v>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>one 'rail:delay_s' entry per line</t>
-        </is>
-      </c>
+      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1476,12 +1474,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>voltage_tolerance_pct</t>
+          <t>impedance_min_ohm</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1497,9 +1495,7 @@
       <c r="G27" t="n">
         <v>0</v>
       </c>
-      <c r="H27" t="n">
-        <v>5</v>
-      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="b">
         <v>1</v>
@@ -1519,17 +1515,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>impedance_min_ohm</t>
+          <t>sample_rate_hz</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1000</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -1538,9 +1534,11 @@
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H28" t="n">
+        <v>250000</v>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="b">
         <v>1</v>
@@ -1560,17 +1558,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>sample_rate_hz</t>
+          <t>pre_trigger_s</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1000</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1578,12 +1576,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G29" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" t="n">
-        <v>250000</v>
-      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="b">
         <v>1</v>
@@ -1603,12 +1597,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>pre_trigger_s</t>
+          <t>post_trigger_s</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>-0.5</t>
+          <t>6.0</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1642,17 +1636,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>post_trigger_s</t>
+          <t>anomaly_policy</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>6.0</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -1662,7 +1656,11 @@
       </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>stop/warn</t>
+        </is>
+      </c>
       <c r="J31" t="b">
         <v>1</v>
       </c>
@@ -1671,41 +1669,25 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Build Impedance/Voltage/Power rails up sequence</t>
+          <t>Build Clocks</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>rails</t>
+          <t>clocks</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>anomaly_policy</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>stop</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>stop/warn</t>
-        </is>
-      </c>
+      <c r="I32" t="inlineStr"/>
       <c r="J32" t="b">
         <v>1</v>
       </c>
@@ -1724,19 +1706,36 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
+          <t>clocks</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CLK1:32768:2
+CLK2:4000000:2</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="b">
         <v>1</v>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>one 'name:freq_hz:tolerance_pct' per line</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1751,36 +1750,35 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>clocks</t>
+          <t>stabilize_ms</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CLK1:32768:2
-CLK2:4000000:2</t>
+          <t>100</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>10000</v>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="b">
         <v>1</v>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>one 'name:freq_hz:tolerance_pct' per line</t>
-        </is>
-      </c>
+      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1795,17 +1793,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>stabilize_ms</t>
+          <t>drift_check</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1813,12 +1811,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G35" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" t="n">
-        <v>10000</v>
-      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="b">
         <v>1</v>
@@ -1838,12 +1832,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>drift_check</t>
+          <t>multi_domain_check</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1867,34 +1861,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Build Clocks</t>
+          <t>Build GPIOs</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>clocks</t>
+          <t>gpios</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>multi_domain_check</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
@@ -1916,19 +1898,36 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
+          <t>groups</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>GPIO0:TP_G0.1:out:none
+GPIO1:TP_G1.1:in:pullup</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="b">
         <v>1</v>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>one 'name:pin:mode:pull' per line</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1943,36 +1942,35 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>groups</t>
+          <t>level_threshold_v</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>GPIO0:TP_G0.1:out:none
-GPIO1:TP_G1.1:in:pullup</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>5</v>
+      </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="b">
         <v>1</v>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>one 'name:pin:mode:pull' per line</t>
-        </is>
-      </c>
+      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1987,17 +1985,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>level_threshold_v</t>
+          <t>exception_check</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -2005,12 +2003,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G40" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" t="n">
-        <v>5</v>
-      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="b">
         <v>1</v>
@@ -2020,34 +2014,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Build GPIOs</t>
+          <t>Configure Programmer/Debugger</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>gpios</t>
+          <t>programmer</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>exception_check</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
@@ -2069,15 +2051,31 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
+          <t>protocol</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SWD</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>choice</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>SWD/JTAG</t>
+        </is>
+      </c>
       <c r="J42" t="b">
         <v>1</v>
       </c>
@@ -2096,17 +2094,17 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>protocol</t>
+          <t>speed_khz</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>SWD</t>
+          <t>4000</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2114,13 +2112,13 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>SWD/JTAG</t>
-        </is>
-      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I43" t="inlineStr"/>
       <c r="J43" t="b">
         <v>1</v>
       </c>
@@ -2139,12 +2137,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>speed_khz</t>
+          <t>timeout_ms</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>4000</t>
+          <t>30000</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2158,10 +2156,10 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="H44" t="n">
-        <v>100000</v>
+        <v>600000</v>
       </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="b">
@@ -2182,17 +2180,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>timeout_ms</t>
+          <t>flash_address</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>30000</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2200,12 +2198,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G45" t="n">
-        <v>100</v>
-      </c>
-      <c r="H45" t="n">
-        <v>600000</v>
-      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="b">
         <v>1</v>
@@ -2225,17 +2219,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>flash_address</t>
+          <t>retries</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>0x0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2243,8 +2237,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>10</v>
+      </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="b">
         <v>1</v>
@@ -2264,17 +2262,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>retries</t>
+          <t>log_level</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>info</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2282,13 +2280,13 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>10</v>
-      </c>
-      <c r="I47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>debug/info/warning/error</t>
+        </is>
+      </c>
       <c r="J47" t="b">
         <v>1</v>
       </c>
@@ -2297,41 +2295,25 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Configure Programmer/Debugger</t>
+          <t>Configure Peripherals</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>programmer</t>
+          <t>peripherals</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>log_level</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>info</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>choice</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>debug/info/warning/error</t>
-        </is>
-      </c>
+      <c r="I48" t="inlineStr"/>
       <c r="J48" t="b">
         <v>1</v>
       </c>
@@ -2350,12 +2332,20 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>__module__</t>
+          <t>wifi_ssid</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
-      <c r="F49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr"/>
@@ -2377,7 +2367,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>wifi_ssid</t>
+          <t>wifi_password</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -2412,7 +2402,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>wifi_password</t>
+          <t>bt_mac</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -2447,13 +2437,17 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>bt_mac</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr"/>
+          <t>uart_baud</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>115200</t>
+        </is>
+      </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2461,8 +2455,12 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
+      <c r="G52" t="n">
+        <v>9600</v>
+      </c>
+      <c r="H52" t="n">
+        <v>921600</v>
+      </c>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="b">
         <v>1</v>
@@ -2482,17 +2480,13 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>uart_baud</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>115200</t>
-        </is>
-      </c>
+          <t>i2c_addr</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2500,12 +2494,8 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G53" t="n">
-        <v>9600</v>
-      </c>
-      <c r="H53" t="n">
-        <v>921600</v>
-      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="b">
         <v>1</v>
@@ -2525,13 +2515,13 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>i2c_addr</t>
+          <t>spi_speed_hz</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2539,7 +2529,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="b">
@@ -2560,13 +2552,13 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>spi_speed_hz</t>
+          <t>adc_ref_v</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>int</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2575,9 +2567,11 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="H55" t="n">
+        <v>10</v>
+      </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="b">
         <v>1</v>
@@ -2597,13 +2591,13 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>adc_ref_v</t>
+          <t>init_sequence</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2611,56 +2605,44 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G56" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" t="n">
-        <v>10</v>
-      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="b">
         <v>1</v>
       </c>
-      <c r="K56" t="inlineStr"/>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>one init step per line</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Configure Peripherals</t>
+          <t>Parse Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>peripherals</t>
+          <t>fct_parse</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>init_sequence</t>
+          <t>__module__</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="b">
-        <v>1</v>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>one init step per line</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2675,12 +2657,24 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
+          <t>spec_file</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>specs/fct_FRDM-IMX93_placeholder.json</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr"/>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
@@ -2702,22 +2696,22 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>spec_file</t>
+          <t>interfaces</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>specs/fct_FRDM-IMX93_placeholder.json</t>
+          <t>(FCT skipped - ICT-only plan)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G59" t="inlineStr"/>
@@ -2726,7 +2720,11 @@
       <c r="J59" t="b">
         <v>0</v>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>one interface per line</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2741,7 +2739,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>interfaces</t>
+          <t>protocols</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2767,7 +2765,7 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>one interface per line</t>
+          <t>one protocol per line</t>
         </is>
       </c>
     </row>
@@ -2784,14 +2782,10 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>protocols</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>(FCT skipped - ICT-only plan)</t>
-        </is>
-      </c>
+          <t>custom_checks</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr">
         <is>
           <t>text</t>
@@ -2810,48 +2804,36 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>one protocol per line</t>
+          <t>one check rule per line</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Parse Func/Interface for FCT</t>
+          <t>Build Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>fct_parse</t>
+          <t>fct_build</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>custom_checks</t>
+          <t>__module__</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="b">
         <v>0</v>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>one check rule per line</t>
-        </is>
-      </c>
+      <c r="K62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2866,19 +2848,35 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
+          <t>flow_steps</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>(FCT skipped - ICT-only plan)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="b">
         <v>0</v>
       </c>
-      <c r="K63" t="inlineStr"/>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>one flow step per line</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2893,35 +2891,35 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>flow_steps</t>
+          <t>yield_threshold_pct</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>(FCT skipped - ICT-only plan)</t>
+          <t>98.0</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+      <c r="H64" t="n">
+        <v>100</v>
+      </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="b">
         <v>0</v>
       </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>one flow step per line</t>
-        </is>
-      </c>
+      <c r="K64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2936,17 +2934,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>yield_threshold_pct</t>
+          <t>exception_branch</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>98.0</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2954,13 +2952,13 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G65" t="n">
-        <v>0</v>
-      </c>
-      <c r="H65" t="n">
-        <v>100</v>
-      </c>
-      <c r="I65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>continue/stop</t>
+        </is>
+      </c>
       <c r="J65" t="b">
         <v>0</v>
       </c>
@@ -2979,17 +2977,13 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>exception_branch</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>stop</t>
-        </is>
-      </c>
+          <t>case_link</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2999,11 +2993,7 @@
       </c>
       <c r="G66" t="inlineStr"/>
       <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>continue/stop</t>
-        </is>
-      </c>
+      <c r="I66" t="inlineStr"/>
       <c r="J66" t="b">
         <v>0</v>
       </c>
@@ -3012,35 +3002,27 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Build Func/Interface for FCT</t>
+          <t>Validate Full Test Sequence</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>fct_build</t>
+          <t>validate_sequence</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>case_link</t>
+          <t>__module__</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
       <c r="J67" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K67" t="inlineStr"/>
     </row>
@@ -3057,12 +3039,24 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
+          <t>resource_conflict_check</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G68" t="inlineStr"/>
       <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr"/>
@@ -3084,7 +3078,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>resource_conflict_check</t>
+          <t>param_range_check</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3123,7 +3117,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>param_range_check</t>
+          <t>dependency_check</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3152,34 +3146,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Validate Full Test Sequence</t>
+          <t>Preview &amp; Export YAML</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>validate_sequence</t>
+          <t>preview_export</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>dependency_check</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+          <t>__module__</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
@@ -3201,19 +3183,35 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
+          <t>export_dir</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>config/plans</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="b">
         <v>1</v>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>project config folder for the exported YAML</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3228,17 +3226,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>export_dir</t>
+          <t>include_disabled</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>config/plans</t>
+          <t>False</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3252,50 +3250,7 @@
       <c r="J73" t="b">
         <v>1</v>
       </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>project config folder for the exported YAML</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Preview &amp; Export YAML</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>preview_export</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>include_disabled</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="b">
-        <v>1</v>
-      </c>
-      <c r="K74" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(yaml-build): 7:3 splitter default, FCT parse block removed, block 08 renamed, card marks (star on OK, check after validation pass)
</commit_message>
<xml_diff>
--- a/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
+++ b/config/examples/Plan_10342_FRDM-IMX93_v1.0.0.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K73"/>
+  <dimension ref="A1:K68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,16 +492,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="b">
         <v>1</v>
       </c>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -534,9 +527,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="b">
         <v>1</v>
       </c>
@@ -577,9 +567,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="b">
         <v>1</v>
       </c>
@@ -620,9 +607,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="b">
         <v>1</v>
       </c>
@@ -663,9 +647,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="b">
         <v>1</v>
       </c>
@@ -706,8 +687,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>EVT (Proto-1)/DVT (Proto-2)/PVT (Pilot-1)/Ramp-up (Pilot-2)/MP (Production)/Deviation (DRQ)/R&amp;R (Return&amp;Rework)/Customized</t>
@@ -716,7 +695,6 @@
       <c r="J7" t="b">
         <v>1</v>
       </c>
-      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -749,9 +727,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="b">
         <v>1</v>
       </c>
@@ -792,9 +767,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="b">
         <v>1</v>
       </c>
@@ -820,16 +792,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="b">
         <v>1</v>
       </c>
-      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -862,13 +827,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="b">
         <v>1</v>
       </c>
-      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -886,7 +847,6 @@
           <t>power_dont_test</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>text</t>
@@ -897,13 +857,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="b">
         <v>1</v>
       </c>
-      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -921,16 +877,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="b">
         <v>1</v>
       </c>
-      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -963,9 +912,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="b">
         <v>1</v>
       </c>
@@ -1006,9 +952,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="b">
         <v>1</v>
       </c>
@@ -1034,7 +977,6 @@
           <t>dmm_visa</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>str</t>
@@ -1045,9 +987,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="b">
         <v>1</v>
       </c>
@@ -1073,7 +1012,6 @@
           <t>channel_alloc</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>text</t>
@@ -1084,9 +1022,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="b">
         <v>1</v>
       </c>
@@ -1127,13 +1062,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="b">
         <v>1</v>
       </c>
-      <c r="K18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1151,16 +1082,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="b">
         <v>1</v>
       </c>
-      <c r="K19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1199,11 +1123,9 @@
       <c r="H20" t="n">
         <v>60</v>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="b">
         <v>1</v>
       </c>
-      <c r="K20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1242,11 +1164,9 @@
       <c r="H21" t="n">
         <v>12.5</v>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="b">
         <v>1</v>
       </c>
-      <c r="K21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1285,11 +1205,9 @@
       <c r="H22" t="n">
         <v>60000</v>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="b">
         <v>1</v>
       </c>
-      <c r="K22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1328,11 +1246,9 @@
       <c r="H23" t="n">
         <v>60000</v>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="b">
         <v>1</v>
       </c>
-      <c r="K23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1365,13 +1281,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="b">
         <v>1</v>
       </c>
-      <c r="K24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1406,9 +1318,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="b">
         <v>1</v>
       </c>
@@ -1455,11 +1364,9 @@
       <c r="H26" t="n">
         <v>5</v>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="b">
         <v>1</v>
       </c>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1495,12 +1402,9 @@
       <c r="G27" t="n">
         <v>0</v>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="b">
         <v>1</v>
       </c>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1539,11 +1443,9 @@
       <c r="H28" t="n">
         <v>250000</v>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="b">
         <v>1</v>
       </c>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1576,13 +1478,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="b">
         <v>1</v>
       </c>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1615,13 +1513,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="b">
         <v>1</v>
       </c>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1654,8 +1548,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>stop/warn</t>
@@ -1664,7 +1556,6 @@
       <c r="J31" t="b">
         <v>1</v>
       </c>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1682,16 +1573,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="b">
         <v>1</v>
       </c>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1725,9 +1609,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="b">
         <v>1</v>
       </c>
@@ -1774,11 +1655,9 @@
       <c r="H34" t="n">
         <v>10000</v>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="b">
         <v>1</v>
       </c>
-      <c r="K34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1811,13 +1690,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="b">
         <v>1</v>
       </c>
-      <c r="K35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1850,13 +1725,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="b">
         <v>1</v>
       </c>
-      <c r="K36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1874,16 +1745,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="b">
         <v>1</v>
       </c>
-      <c r="K37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1917,9 +1781,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="b">
         <v>1</v>
       </c>
@@ -1966,11 +1827,9 @@
       <c r="H39" t="n">
         <v>5</v>
       </c>
-      <c r="I39" t="inlineStr"/>
       <c r="J39" t="b">
         <v>1</v>
       </c>
-      <c r="K39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2003,13 +1862,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
       <c r="J40" t="b">
         <v>1</v>
       </c>
-      <c r="K40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2027,16 +1882,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
       <c r="J41" t="b">
         <v>1</v>
       </c>
-      <c r="K41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2069,8 +1917,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>SWD/JTAG</t>
@@ -2079,7 +1925,6 @@
       <c r="J42" t="b">
         <v>1</v>
       </c>
-      <c r="K42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2118,11 +1963,9 @@
       <c r="H43" t="n">
         <v>100000</v>
       </c>
-      <c r="I43" t="inlineStr"/>
       <c r="J43" t="b">
         <v>1</v>
       </c>
-      <c r="K43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2161,11 +2004,9 @@
       <c r="H44" t="n">
         <v>600000</v>
       </c>
-      <c r="I44" t="inlineStr"/>
       <c r="J44" t="b">
         <v>1</v>
       </c>
-      <c r="K44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2198,13 +2039,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
       <c r="J45" t="b">
         <v>1</v>
       </c>
-      <c r="K45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2243,11 +2080,9 @@
       <c r="H46" t="n">
         <v>10</v>
       </c>
-      <c r="I46" t="inlineStr"/>
       <c r="J46" t="b">
         <v>1</v>
       </c>
-      <c r="K46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2280,8 +2115,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>debug/info/warning/error</t>
@@ -2290,7 +2123,6 @@
       <c r="J47" t="b">
         <v>1</v>
       </c>
-      <c r="K47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2308,16 +2140,9 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
       <c r="J48" t="b">
         <v>1</v>
       </c>
-      <c r="K48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2335,7 +2160,6 @@
           <t>wifi_ssid</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
           <t>str</t>
@@ -2346,13 +2170,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
       <c r="J49" t="b">
         <v>1</v>
       </c>
-      <c r="K49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2370,7 +2190,6 @@
           <t>wifi_password</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
           <t>str</t>
@@ -2381,13 +2200,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
       <c r="J50" t="b">
         <v>1</v>
       </c>
-      <c r="K50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2405,7 +2220,6 @@
           <t>bt_mac</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>str</t>
@@ -2416,13 +2230,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
       <c r="J51" t="b">
         <v>1</v>
       </c>
-      <c r="K51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2461,11 +2271,9 @@
       <c r="H52" t="n">
         <v>921600</v>
       </c>
-      <c r="I52" t="inlineStr"/>
       <c r="J52" t="b">
         <v>1</v>
       </c>
-      <c r="K52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2483,7 +2291,6 @@
           <t>i2c_addr</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>str</t>
@@ -2494,13 +2301,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
       <c r="J53" t="b">
         <v>1</v>
       </c>
-      <c r="K53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2518,7 +2321,6 @@
           <t>spi_speed_hz</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>int</t>
@@ -2532,12 +2334,9 @@
       <c r="G54" t="n">
         <v>1</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
       <c r="J54" t="b">
         <v>1</v>
       </c>
-      <c r="K54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2555,7 +2354,6 @@
           <t>adc_ref_v</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
           <t>float</t>
@@ -2572,11 +2370,9 @@
       <c r="H55" t="n">
         <v>10</v>
       </c>
-      <c r="I55" t="inlineStr"/>
       <c r="J55" t="b">
         <v>1</v>
       </c>
-      <c r="K55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2594,7 +2390,6 @@
           <t>init_sequence</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
           <t>text</t>
@@ -2605,9 +2400,6 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
       <c r="J56" t="b">
         <v>1</v>
       </c>
@@ -2620,12 +2412,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Parse Func/Interface for FCT</t>
+          <t>Build Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>fct_parse</t>
+          <t>fct_build</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2633,41 +2425,34 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
       <c r="J57" t="b">
         <v>0</v>
       </c>
-      <c r="K57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Parse Func/Interface for FCT</t>
+          <t>Build Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>fct_parse</t>
+          <t>fct_build</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>spec_file</t>
+          <t>flow_steps</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>specs/fct_FRDM-IMX93_placeholder.json</t>
+          <t>(FCT skipped - ICT-only plan)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>text</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2675,38 +2460,39 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
       <c r="J58" t="b">
         <v>0</v>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>one flow step per line</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Parse Func/Interface for FCT</t>
+          <t>Build Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>fct_parse</t>
+          <t>fct_build</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>interfaces</t>
+          <t>yield_threshold_pct</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>(FCT skipped - ICT-only plan)</t>
+          <t>98.0</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>float</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2714,42 +2500,40 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="n">
+        <v>100</v>
+      </c>
       <c r="J59" t="b">
         <v>0</v>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>one interface per line</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Parse Func/Interface for FCT</t>
+          <t>Build Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>fct_parse</t>
+          <t>fct_build</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>protocols</t>
+          <t>exception_branch</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>(FCT skipped - ICT-only plan)</t>
+          <t>stop</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>choice</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2757,38 +2541,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>continue/stop</t>
+        </is>
+      </c>
       <c r="J60" t="b">
         <v>0</v>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>one protocol per line</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Parse Func/Interface for FCT</t>
+          <t>Build Func/Interface for FCT</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>fct_parse</t>
+          <t>fct_build</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>custom_checks</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+          <t>case_link</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>str</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2796,27 +2576,19 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
       <c r="J61" t="b">
         <v>0</v>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>one check rule per line</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Build Func/Interface for FCT</t>
+          <t>Validate Full Test Sequence</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>fct_build</t>
+          <t>validate_sequence</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2824,84 +2596,69 @@
           <t>__module__</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
       <c r="J62" t="b">
-        <v>0</v>
-      </c>
-      <c r="K62" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Build Func/Interface for FCT</t>
+          <t>Validate Full Test Sequence</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>fct_build</t>
+          <t>validate_sequence</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>flow_steps</t>
+          <t>resource_conflict_check</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>(FCT skipped - ICT-only plan)</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
       <c r="J63" t="b">
-        <v>0</v>
-      </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>one flow step per line</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Build Func/Interface for FCT</t>
+          <t>Validate Full Test Sequence</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>fct_build</t>
+          <t>validate_sequence</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>yield_threshold_pct</t>
+          <t>param_range_check</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>98.0</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>float</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2909,42 +2666,34 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G64" t="n">
-        <v>0</v>
-      </c>
-      <c r="H64" t="n">
-        <v>100</v>
-      </c>
-      <c r="I64" t="inlineStr"/>
       <c r="J64" t="b">
-        <v>0</v>
-      </c>
-      <c r="K64" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Build Func/Interface for FCT</t>
+          <t>Validate Full Test Sequence</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>fct_build</t>
+          <t>validate_sequence</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>exception_branch</t>
+          <t>dependency_check</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>True</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>choice</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2952,99 +2701,89 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>continue/stop</t>
-        </is>
-      </c>
       <c r="J65" t="b">
-        <v>0</v>
-      </c>
-      <c r="K65" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Build Func/Interface for FCT</t>
+          <t>Preview &amp; Export YAML</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>fct_build</t>
+          <t>preview_export</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>case_link</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr"/>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
+          <t>__module__</t>
+        </is>
+      </c>
       <c r="J66" t="b">
-        <v>0</v>
-      </c>
-      <c r="K66" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Validate Full Test Sequence</t>
+          <t>Preview &amp; Export YAML</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>validate_sequence</t>
+          <t>preview_export</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
+          <t>export_dir</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>config/plans</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="J67" t="b">
         <v>1</v>
       </c>
-      <c r="K67" t="inlineStr"/>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>project config folder for the exported YAML</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Validate Full Test Sequence</t>
+          <t>Preview &amp; Export YAML</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>validate_sequence</t>
+          <t>preview_export</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>resource_conflict_check</t>
+          <t>include_disabled</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3057,200 +2796,9 @@
           <t>no</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
-      <c r="I68" t="inlineStr"/>
       <c r="J68" t="b">
         <v>1</v>
       </c>
-      <c r="K68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Validate Full Test Sequence</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>validate_sequence</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>param_range_check</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="b">
-        <v>1</v>
-      </c>
-      <c r="K69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Validate Full Test Sequence</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>validate_sequence</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>dependency_check</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="b">
-        <v>1</v>
-      </c>
-      <c r="K70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Preview &amp; Export YAML</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>preview_export</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>__module__</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
-      <c r="E71" t="inlineStr"/>
-      <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="b">
-        <v>1</v>
-      </c>
-      <c r="K71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Preview &amp; Export YAML</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>preview_export</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>export_dir</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>config/plans</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="b">
-        <v>1</v>
-      </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>project config folder for the exported YAML</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Preview &amp; Export YAML</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>preview_export</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>include_disabled</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>bool</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="b">
-        <v>1</v>
-      </c>
-      <c r="K73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>